<commit_message>
robustness glm (richness and offset(richness))
</commit_message>
<xml_diff>
--- a/Data/Processed/GLM_results.xlsx
+++ b/Data/Processed/GLM_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\OneDrive\Desktop\Collabs\Extinction_dynamics_Iberic\Data\Processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88C53B72-CF10-4FBB-8D07-C392DF12C19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34952A3-DB49-4617-B97E-74AC37F4F9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{74ED5B23-4F77-4FB6-972B-07F52B9703B8}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="17925" windowHeight="15585" xr2:uid="{74ED5B23-4F77-4FB6-972B-07F52B9703B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -188,15 +188,21 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -204,32 +210,177 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -560,34 +711,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="11" t="s">
         <v>6</v>
       </c>
       <c r="K1" s="1"/>
@@ -619,39 +770,39 @@
       <c r="AK1" s="1"/>
     </row>
     <row r="2" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="20">
         <v>1767.6</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="21">
         <f>D2-D4</f>
         <v>1.8999999999998636</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G2" s="22">
         <v>1E-3</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H2" s="22">
         <v>0.7</v>
       </c>
-      <c r="I2" s="6">
+      <c r="I2" s="22">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="19">
         <v>1.4E-3</v>
       </c>
-      <c r="K2" s="6"/>
-      <c r="L2" s="4"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="2"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
@@ -679,26 +830,26 @@
       <c r="AK2" s="1"/>
     </row>
     <row r="3" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="6" t="s">
+      <c r="A3" s="12"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="22">
         <v>-0.379</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="22">
         <v>0.23</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="22">
         <v>0.31</v>
       </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="4"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="2"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
@@ -726,34 +877,34 @@
       <c r="AK3" s="1"/>
     </row>
     <row r="4" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="7" t="s">
+      <c r="A4" s="12"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="25">
         <v>1765.7</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="25">
         <v>0</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="25">
         <v>-0.43</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="25">
         <v>0.14199999999999999</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="25">
         <v>0.28999999999999998</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="22">
         <v>1.4E-3</v>
       </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="4"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="2"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
@@ -781,35 +932,35 @@
       <c r="AK4" s="1"/>
     </row>
     <row r="5" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="6" t="s">
+      <c r="A5" s="12"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="22">
         <v>1767.2</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="22">
         <f>D5-D4</f>
         <v>1.5</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="22">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="22">
         <v>0.32</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="22">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="4"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="2"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
@@ -837,35 +988,35 @@
       <c r="AK5" s="1"/>
     </row>
     <row r="6" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="6" t="s">
+      <c r="A6" s="12"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="22">
         <v>1766.2</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="22">
         <f>D6-D4</f>
         <v>0.5</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="4"/>
+      <c r="F6" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="3"/>
+      <c r="L6" s="2"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
@@ -893,17 +1044,17 @@
       <c r="AK6" s="1"/>
     </row>
     <row r="7" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="16">
         <v>1767.4</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <f>D7-D9</f>
         <v>1.7000000000000455</v>
       </c>
@@ -919,11 +1070,11 @@
       <c r="I7" s="6">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="12">
         <v>1.5E-3</v>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="4"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="2"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
@@ -951,10 +1102,10 @@
       <c r="AK7" s="1"/>
     </row>
     <row r="8" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
       <c r="E8" s="5"/>
       <c r="F8" s="6" t="s">
         <v>19</v>
@@ -968,9 +1119,9 @@
       <c r="I8" s="6">
         <v>0.33</v>
       </c>
-      <c r="J8" s="5"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="4"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="2"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
@@ -998,8 +1149,8 @@
       <c r="AK8" s="1"/>
     </row>
     <row r="9" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="12"/>
       <c r="C9" s="7" t="s">
         <v>15</v>
       </c>
@@ -1024,8 +1175,8 @@
       <c r="J9" s="7">
         <v>1.2999999999999999E-3</v>
       </c>
-      <c r="K9" s="6"/>
-      <c r="L9" s="4"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="2"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
@@ -1053,8 +1204,8 @@
       <c r="AK9" s="1"/>
     </row>
     <row r="10" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
+      <c r="A10" s="12"/>
+      <c r="B10" s="12"/>
       <c r="C10" s="6" t="s">
         <v>11</v>
       </c>
@@ -1080,8 +1231,8 @@
       <c r="J10" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="K10" s="6"/>
-      <c r="L10" s="4"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="2"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
@@ -1109,8 +1260,8 @@
       <c r="AK10" s="1"/>
     </row>
     <row r="11" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="12"/>
       <c r="C11" s="6" t="s">
         <v>13</v>
       </c>
@@ -1136,8 +1287,8 @@
       <c r="J11" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="6"/>
-      <c r="L11" s="4"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="2"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
@@ -1165,37 +1316,37 @@
       <c r="AK11" s="1"/>
     </row>
     <row r="12" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="12"/>
+      <c r="B12" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="27">
         <v>1766.8</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="21">
         <f>D12-D15</f>
         <v>1.5999999999999091</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="22">
         <v>1.6E-2</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="22">
         <v>0.34</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I12" s="22">
         <v>0.02</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="19">
         <v>1.8E-3</v>
       </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="4"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="2"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
@@ -1223,26 +1374,26 @@
       <c r="AK12" s="1"/>
     </row>
     <row r="13" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="6" t="s">
+      <c r="A13" s="12"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="6">
+      <c r="G13" s="22">
         <v>-0.22</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="22">
         <v>0.53</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="22">
         <v>0.35</v>
       </c>
-      <c r="J13" s="5"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="4"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="2"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
@@ -1270,35 +1421,35 @@
       <c r="AK13" s="1"/>
     </row>
     <row r="14" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="6" t="s">
+      <c r="A14" s="12"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="22">
         <v>1765.7</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="22">
         <f>D14-D15</f>
         <v>0.5</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="6">
+      <c r="G14" s="22">
         <v>-0.43</v>
       </c>
-      <c r="H14" s="6">
+      <c r="H14" s="22">
         <v>0.14199999999999999</v>
       </c>
-      <c r="I14" s="6">
+      <c r="I14" s="22">
         <v>0.28999999999999998</v>
       </c>
-      <c r="J14" s="6">
+      <c r="J14" s="22">
         <v>1.4E-3</v>
       </c>
-      <c r="K14" s="6"/>
-      <c r="L14" s="4"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="2"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
@@ -1326,34 +1477,34 @@
       <c r="AK14" s="1"/>
     </row>
     <row r="15" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="7" t="s">
+      <c r="A15" s="12"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="25">
         <v>1765.2</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="22">
         <v>0</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="25">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="25">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="25">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="25">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="K15" s="6"/>
-      <c r="L15" s="4"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="2"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
@@ -1381,35 +1532,35 @@
       <c r="AK15" s="1"/>
     </row>
     <row r="16" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="6" t="s">
+      <c r="A16" s="12"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="22">
         <v>1766.2</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="22">
         <f>D16-D15</f>
         <v>1</v>
       </c>
-      <c r="F16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K16" s="6"/>
-      <c r="L16" s="4"/>
+      <c r="F16" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I16" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J16" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="K16" s="3"/>
+      <c r="L16" s="2"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
@@ -1437,19 +1588,19 @@
       <c r="AK16" s="1"/>
     </row>
     <row r="17" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="16">
         <v>1190.7</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="16">
         <f>D17-D20</f>
         <v>1.9000000000000909</v>
       </c>
@@ -1465,11 +1616,11 @@
       <c r="I17" s="6">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="12">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="K17" s="6"/>
-      <c r="L17" s="4"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="2"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
@@ -1497,11 +1648,11 @@
       <c r="AK17" s="1"/>
     </row>
     <row r="18" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
       <c r="F18" s="6" t="s">
         <v>19</v>
       </c>
@@ -1514,9 +1665,9 @@
       <c r="I18" s="6">
         <v>0.45</v>
       </c>
-      <c r="J18" s="5"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="4"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="2"/>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
@@ -1544,8 +1695,8 @@
       <c r="AK18" s="1"/>
     </row>
     <row r="19" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
       <c r="C19" s="6" t="s">
         <v>15</v>
       </c>
@@ -1571,8 +1722,8 @@
       <c r="J19" s="6">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="K19" s="6"/>
-      <c r="L19" s="4"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="2"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
@@ -1600,8 +1751,8 @@
       <c r="AK19" s="1"/>
     </row>
     <row r="20" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
       <c r="C20" s="7" t="s">
         <v>11</v>
       </c>
@@ -1626,8 +1777,8 @@
       <c r="J20" s="7">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="K20" s="6"/>
-      <c r="L20" s="4"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="2"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
@@ -1655,8 +1806,8 @@
       <c r="AK20" s="1"/>
     </row>
     <row r="21" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
       <c r="C21" s="6" t="s">
         <v>13</v>
       </c>
@@ -1682,8 +1833,8 @@
       <c r="J21" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K21" s="6"/>
-      <c r="L21" s="4"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="2"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
@@ -1711,37 +1862,37 @@
       <c r="AK21" s="1"/>
     </row>
     <row r="22" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5" t="s">
+      <c r="A22" s="12"/>
+      <c r="B22" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="20">
         <v>1190.5999999999999</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="20">
         <f>D22-D25</f>
         <v>2</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="G22" s="6">
+      <c r="G22" s="22">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="22">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="22">
         <v>1.6E-2</v>
       </c>
-      <c r="J22" s="5">
+      <c r="J22" s="19">
         <v>6.6E-3</v>
       </c>
-      <c r="K22" s="6"/>
-      <c r="L22" s="4"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="2"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
@@ -1769,26 +1920,26 @@
       <c r="AK22" s="1"/>
     </row>
     <row r="23" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="6" t="s">
+      <c r="A23" s="12"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="22">
         <v>-1E-3</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="22">
         <v>0.99</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="22">
         <v>0.46</v>
       </c>
-      <c r="J23" s="5"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="4"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="2"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
@@ -1816,35 +1967,35 @@
       <c r="AK23" s="1"/>
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="6" t="s">
+      <c r="A24" s="12"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="22">
         <v>1194.4000000000001</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="22">
         <f>D24-D25</f>
         <v>5.8000000000001819</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="6">
+      <c r="G24" s="22">
         <v>-0.61</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="22">
         <v>0.185</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="22">
         <v>0.46</v>
       </c>
-      <c r="J24" s="6">
+      <c r="J24" s="22">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
@@ -1872,30 +2023,30 @@
       <c r="AK24" s="1"/>
     </row>
     <row r="25" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="7" t="s">
+      <c r="A25" s="12"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="25">
         <v>1188.5999999999999</v>
       </c>
-      <c r="E25" s="7">
+      <c r="E25" s="25">
         <v>0</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="G25" s="7">
+      <c r="G25" s="25">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="H25" s="7" t="s">
+      <c r="H25" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="I25" s="7">
+      <c r="I25" s="25">
         <v>0.01</v>
       </c>
-      <c r="J25" s="7">
+      <c r="J25" s="25">
         <v>6.6E-3</v>
       </c>
       <c r="K25" s="1"/>
@@ -1927,30 +2078,30 @@
       <c r="AK25" s="1"/>
     </row>
     <row r="26" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="6" t="s">
+      <c r="A26" s="12"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="22">
         <v>1194.4000000000001</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="22">
         <v>5.8</v>
       </c>
-      <c r="F26" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J26" s="8" t="s">
+      <c r="F26" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="G26" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="H26" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J26" s="26" t="s">
         <v>20</v>
       </c>
       <c r="K26" s="1"/>
@@ -1982,17 +2133,17 @@
       <c r="AK26" s="1"/>
     </row>
     <row r="27" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5" t="s">
+      <c r="A27" s="12"/>
+      <c r="B27" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="16">
         <v>1190.3</v>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="16">
         <f>D27-D30</f>
         <v>4.7999999999999545</v>
       </c>
@@ -2008,7 +2159,7 @@
       <c r="I27" s="6">
         <v>0.02</v>
       </c>
-      <c r="J27" s="5">
+      <c r="J27" s="14">
         <v>6.7999999999999996E-3</v>
       </c>
       <c r="K27" s="1"/>
@@ -2040,24 +2191,24 @@
       <c r="AK27" s="1"/>
     </row>
     <row r="28" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="6" t="s">
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="G28" s="6">
+      <c r="G28" s="18">
         <v>0.17</v>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="18">
         <v>0.72</v>
       </c>
-      <c r="I28" s="6">
+      <c r="I28" s="18">
         <v>0.48</v>
       </c>
-      <c r="J28" s="5"/>
+      <c r="J28" s="15"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -2087,9 +2238,9 @@
       <c r="AK28" s="1"/>
     </row>
     <row r="29" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="6" t="s">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="9" t="s">
         <v>15</v>
       </c>
       <c r="D29" s="6">
@@ -2143,9 +2294,9 @@
       <c r="AK29" s="1"/>
     </row>
     <row r="30" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="7" t="s">
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="10" t="s">
         <v>11</v>
       </c>
       <c r="D30" s="7">
@@ -2198,9 +2349,9 @@
       <c r="AK30" s="1"/>
     </row>
     <row r="31" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="6" t="s">
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="9" t="s">
         <v>13</v>
       </c>
       <c r="D31" s="6">
@@ -2410,16 +2561,12 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J12:J13"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C22:C23"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="J2:J3"/>
@@ -2436,12 +2583,16 @@
     <mergeCell ref="B17:B21"/>
     <mergeCell ref="B22:B26"/>
     <mergeCell ref="B27:B31"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="J27:J28"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
GLM residuals diagnosis and GLM summary
</commit_message>
<xml_diff>
--- a/Data/Processed/GLM_results.xlsx
+++ b/Data/Processed/GLM_results.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\OneDrive\Desktop\Collabs\Extinction_dynamics_Iberic\Data\Processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F34952A3-DB49-4617-B97E-74AC37F4F9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8F3D3B-CD8E-4968-A831-0A551B63AF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="17925" windowHeight="15585" xr2:uid="{74ED5B23-4F77-4FB6-972B-07F52B9703B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{74ED5B23-4F77-4FB6-972B-07F52B9703B8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Complete" sheetId="1" r:id="rId1"/>
+    <sheet name="summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="25">
   <si>
     <t>Region</t>
   </si>
@@ -188,7 +189,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,6 +199,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -299,19 +306,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -332,16 +333,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -350,37 +354,46 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -711,34 +724,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="9" t="s">
         <v>6</v>
       </c>
       <c r="K1" s="1"/>
@@ -770,35 +783,35 @@
       <c r="AK1" s="1"/>
     </row>
     <row r="2" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="17">
         <v>1767.6</v>
       </c>
-      <c r="E2" s="21">
+      <c r="E2" s="19">
         <f>D2-D4</f>
         <v>1.8999999999998636</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="22">
+      <c r="G2" s="12">
         <v>1E-3</v>
       </c>
-      <c r="H2" s="22">
+      <c r="H2" s="12">
         <v>0.7</v>
       </c>
-      <c r="I2" s="22">
+      <c r="I2" s="12">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="J2" s="19">
+      <c r="J2" s="21">
         <v>1.4E-3</v>
       </c>
       <c r="K2" s="3"/>
@@ -830,24 +843,24 @@
       <c r="AK2" s="1"/>
     </row>
     <row r="3" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="22" t="s">
+      <c r="A3" s="22"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="22">
+      <c r="G3" s="12">
         <v>-0.379</v>
       </c>
-      <c r="H3" s="22">
+      <c r="H3" s="12">
         <v>0.23</v>
       </c>
-      <c r="I3" s="22">
+      <c r="I3" s="12">
         <v>0.31</v>
       </c>
-      <c r="J3" s="19"/>
+      <c r="J3" s="21"/>
       <c r="K3" s="3"/>
       <c r="L3" s="2"/>
       <c r="M3" s="1"/>
@@ -877,30 +890,30 @@
       <c r="AK3" s="1"/>
     </row>
     <row r="4" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A4" s="12"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="25" t="s">
+      <c r="A4" s="22"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="13">
         <v>1765.7</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="13">
         <v>0</v>
       </c>
-      <c r="F4" s="25" t="s">
+      <c r="F4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="13">
         <v>-0.43</v>
       </c>
-      <c r="H4" s="25">
+      <c r="H4" s="13">
         <v>0.14199999999999999</v>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="13">
         <v>0.28999999999999998</v>
       </c>
-      <c r="J4" s="22">
+      <c r="J4" s="13">
         <v>1.4E-3</v>
       </c>
       <c r="K4" s="3"/>
@@ -932,31 +945,31 @@
       <c r="AK4" s="1"/>
     </row>
     <row r="5" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A5" s="12"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="22" t="s">
+      <c r="A5" s="22"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="12">
         <v>1767.2</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="12">
         <f>D5-D4</f>
         <v>1.5</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="12">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="12">
         <v>0.32</v>
       </c>
-      <c r="I5" s="22">
+      <c r="I5" s="12">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="J5" s="22" t="s">
+      <c r="J5" s="12" t="s">
         <v>24</v>
       </c>
       <c r="K5" s="3"/>
@@ -988,31 +1001,31 @@
       <c r="AK5" s="1"/>
     </row>
     <row r="6" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A6" s="12"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="22" t="s">
+      <c r="A6" s="22"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="12">
         <v>1766.2</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="12">
         <f>D6-D4</f>
         <v>0.5</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="26" t="s">
+      <c r="G6" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="26" t="s">
+      <c r="H6" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="26" t="s">
+      <c r="I6" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="26" t="s">
+      <c r="J6" s="14" t="s">
         <v>20</v>
       </c>
       <c r="K6" s="3"/>
@@ -1044,33 +1057,33 @@
       <c r="AK6" s="1"/>
     </row>
     <row r="7" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="15">
         <v>1767.4</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="25">
         <f>D7-D9</f>
         <v>1.7000000000000455</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="4">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="4">
         <v>0.56999999999999995</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="4">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="J7" s="12">
+      <c r="J7" s="22">
         <v>1.5E-3</v>
       </c>
       <c r="K7" s="3"/>
@@ -1102,24 +1115,24 @@
       <c r="AK7" s="1"/>
     </row>
     <row r="8" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="6" t="s">
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="4">
         <v>-0.33</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="4">
         <v>0.32</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="4">
         <v>0.33</v>
       </c>
-      <c r="J8" s="12"/>
+      <c r="J8" s="22"/>
       <c r="K8" s="3"/>
       <c r="L8" s="2"/>
       <c r="M8" s="1"/>
@@ -1149,30 +1162,30 @@
       <c r="AK8" s="1"/>
     </row>
     <row r="9" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="7" t="s">
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="5">
         <v>1765.7</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="5">
         <v>0</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="5">
         <v>-0.43</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="5">
         <v>0.14199999999999999</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="5">
         <v>0.28999999999999998</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="5">
         <v>1.2999999999999999E-3</v>
       </c>
       <c r="K9" s="3"/>
@@ -1204,31 +1217,31 @@
       <c r="AK9" s="1"/>
     </row>
     <row r="10" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="6" t="s">
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>1766.5</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="4">
         <f>D10-D9</f>
         <v>0.79999999999995453</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="4">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="4">
         <v>0.19600000000000001</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="4">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="J10" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K10" s="3"/>
@@ -1260,31 +1273,31 @@
       <c r="AK10" s="1"/>
     </row>
     <row r="11" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="6" t="s">
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="4">
         <v>1766.2</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="4">
         <f>D11-D9</f>
         <v>0.5</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="I11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="J11" s="6" t="s">
         <v>20</v>
       </c>
       <c r="K11" s="3"/>
@@ -1316,33 +1329,33 @@
       <c r="AK11" s="1"/>
     </row>
     <row r="12" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
-      <c r="B12" s="19" t="s">
+      <c r="A12" s="22"/>
+      <c r="B12" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="27">
+      <c r="D12" s="23">
         <v>1766.8</v>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="19">
         <f>D12-D15</f>
         <v>1.5999999999999091</v>
       </c>
-      <c r="F12" s="22" t="s">
+      <c r="F12" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="12">
         <v>1.6E-2</v>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="12">
         <v>0.34</v>
       </c>
-      <c r="I12" s="22">
+      <c r="I12" s="12">
         <v>0.02</v>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="21">
         <v>1.8E-3</v>
       </c>
       <c r="K12" s="3"/>
@@ -1374,24 +1387,24 @@
       <c r="AK12" s="1"/>
     </row>
     <row r="13" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="22" t="s">
+      <c r="A13" s="22"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="12">
         <v>-0.22</v>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="12">
         <v>0.53</v>
       </c>
-      <c r="I13" s="22">
+      <c r="I13" s="12">
         <v>0.35</v>
       </c>
-      <c r="J13" s="19"/>
+      <c r="J13" s="21"/>
       <c r="K13" s="3"/>
       <c r="L13" s="2"/>
       <c r="M13" s="1"/>
@@ -1421,31 +1434,31 @@
       <c r="AK13" s="1"/>
     </row>
     <row r="14" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A14" s="12"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="22" t="s">
+      <c r="A14" s="22"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="12">
         <v>1765.7</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="12">
         <f>D14-D15</f>
         <v>0.5</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G14" s="22">
+      <c r="G14" s="12">
         <v>-0.43</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="12">
         <v>0.14199999999999999</v>
       </c>
-      <c r="I14" s="22">
+      <c r="I14" s="12">
         <v>0.28999999999999998</v>
       </c>
-      <c r="J14" s="22">
+      <c r="J14" s="12">
         <v>1.4E-3</v>
       </c>
       <c r="K14" s="3"/>
@@ -1477,30 +1490,30 @@
       <c r="AK14" s="1"/>
     </row>
     <row r="15" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="25" t="s">
+      <c r="A15" s="22"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="13">
         <v>1765.2</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="12">
         <v>0</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="F15" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="13">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="H15" s="25">
+      <c r="H15" s="13">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="I15" s="25">
+      <c r="I15" s="13">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="J15" s="25">
+      <c r="J15" s="13">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="K15" s="3"/>
@@ -1532,31 +1545,31 @@
       <c r="AK15" s="1"/>
     </row>
     <row r="16" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A16" s="12"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="22" t="s">
+      <c r="A16" s="22"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="12">
         <v>1766.2</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="12">
         <f>D16-D15</f>
         <v>1</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="G16" s="26" t="s">
+      <c r="G16" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="H16" s="26" t="s">
+      <c r="H16" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="I16" s="26" t="s">
+      <c r="I16" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="J16" s="26" t="s">
+      <c r="J16" s="14" t="s">
         <v>20</v>
       </c>
       <c r="K16" s="3"/>
@@ -1588,35 +1601,35 @@
       <c r="AK16" s="1"/>
     </row>
     <row r="17" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="15">
         <v>1190.7</v>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="15">
         <f>D17-D20</f>
         <v>1.9000000000000909</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G17" s="4">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="4">
         <v>1.4E-2</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="4">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="J17" s="12">
+      <c r="J17" s="22">
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="K17" s="3"/>
@@ -1648,24 +1661,24 @@
       <c r="AK17" s="1"/>
     </row>
     <row r="18" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="6" t="s">
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G18" s="6">
+      <c r="G18" s="4">
         <v>-0.17</v>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="4">
         <v>0.71</v>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="4">
         <v>0.45</v>
       </c>
-      <c r="J18" s="12"/>
+      <c r="J18" s="22"/>
       <c r="K18" s="3"/>
       <c r="L18" s="2"/>
       <c r="M18" s="1"/>
@@ -1695,31 +1708,31 @@
       <c r="AK18" s="1"/>
     </row>
     <row r="19" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="6" t="s">
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="4">
         <v>1194.4000000000001</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="4">
         <f>D19-D20</f>
         <v>5.6000000000001364</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="6">
+      <c r="G19" s="4">
         <v>-0.61</v>
       </c>
-      <c r="H19" s="6">
+      <c r="H19" s="4">
         <v>0.185</v>
       </c>
-      <c r="I19" s="6">
+      <c r="I19" s="4">
         <v>0.46</v>
       </c>
-      <c r="J19" s="6">
+      <c r="J19" s="4">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="K19" s="3"/>
@@ -1751,30 +1764,30 @@
       <c r="AK19" s="1"/>
     </row>
     <row r="20" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="7" t="s">
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="5">
         <v>1188.8</v>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="5">
         <v>0</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="5">
         <v>1.4E-2</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="5">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="J20" s="7">
+      <c r="J20" s="5">
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="K20" s="3"/>
@@ -1806,31 +1819,31 @@
       <c r="AK20" s="1"/>
     </row>
     <row r="21" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="6" t="s">
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="4">
         <v>1194.4000000000001</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="4">
         <f>D21-D20</f>
         <v>5.6000000000001364</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="8" t="s">
+      <c r="G21" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H21" s="8" t="s">
+      <c r="H21" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I21" s="8" t="s">
+      <c r="I21" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J21" s="8" t="s">
+      <c r="J21" s="6" t="s">
         <v>20</v>
       </c>
       <c r="K21" s="3"/>
@@ -1862,33 +1875,33 @@
       <c r="AK21" s="1"/>
     </row>
     <row r="22" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A22" s="12"/>
-      <c r="B22" s="19" t="s">
+      <c r="A22" s="22"/>
+      <c r="B22" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="17">
         <v>1190.5999999999999</v>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="17">
         <f>D22-D25</f>
         <v>2</v>
       </c>
-      <c r="F22" s="22" t="s">
+      <c r="F22" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22" s="12">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="H22" s="22">
+      <c r="H22" s="12">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="I22" s="22">
+      <c r="I22" s="12">
         <v>1.6E-2</v>
       </c>
-      <c r="J22" s="19">
+      <c r="J22" s="21">
         <v>6.6E-3</v>
       </c>
       <c r="K22" s="3"/>
@@ -1920,24 +1933,24 @@
       <c r="AK22" s="1"/>
     </row>
     <row r="23" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A23" s="12"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="22" t="s">
+      <c r="A23" s="22"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="22">
+      <c r="G23" s="12">
         <v>-1E-3</v>
       </c>
-      <c r="H23" s="22">
+      <c r="H23" s="12">
         <v>0.99</v>
       </c>
-      <c r="I23" s="22">
+      <c r="I23" s="12">
         <v>0.46</v>
       </c>
-      <c r="J23" s="19"/>
+      <c r="J23" s="21"/>
       <c r="K23" s="3"/>
       <c r="L23" s="2"/>
       <c r="M23" s="1"/>
@@ -1967,31 +1980,31 @@
       <c r="AK23" s="1"/>
     </row>
     <row r="24" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A24" s="12"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="22" t="s">
+      <c r="A24" s="22"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="22">
+      <c r="D24" s="12">
         <v>1194.4000000000001</v>
       </c>
-      <c r="E24" s="22">
+      <c r="E24" s="12">
         <f>D24-D25</f>
         <v>5.8000000000001819</v>
       </c>
-      <c r="F24" s="22" t="s">
+      <c r="F24" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="22">
+      <c r="G24" s="12">
         <v>-0.61</v>
       </c>
-      <c r="H24" s="22">
+      <c r="H24" s="12">
         <v>0.185</v>
       </c>
-      <c r="I24" s="22">
+      <c r="I24" s="12">
         <v>0.46</v>
       </c>
-      <c r="J24" s="22">
+      <c r="J24" s="12">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="K24" s="2"/>
@@ -2023,30 +2036,30 @@
       <c r="AK24" s="1"/>
     </row>
     <row r="25" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="25" t="s">
+      <c r="A25" s="22"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="25">
+      <c r="D25" s="13">
         <v>1188.5999999999999</v>
       </c>
-      <c r="E25" s="25">
+      <c r="E25" s="13">
         <v>0</v>
       </c>
-      <c r="F25" s="25" t="s">
+      <c r="F25" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="G25" s="25">
+      <c r="G25" s="13">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="H25" s="25" t="s">
+      <c r="H25" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I25" s="25">
+      <c r="I25" s="13">
         <v>0.01</v>
       </c>
-      <c r="J25" s="25">
+      <c r="J25" s="13">
         <v>6.6E-3</v>
       </c>
       <c r="K25" s="1"/>
@@ -2078,30 +2091,30 @@
       <c r="AK25" s="1"/>
     </row>
     <row r="26" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A26" s="12"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="22" t="s">
+      <c r="A26" s="22"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D26" s="22">
+      <c r="D26" s="12">
         <v>1194.4000000000001</v>
       </c>
-      <c r="E26" s="22">
+      <c r="E26" s="12">
         <v>5.8</v>
       </c>
-      <c r="F26" s="26" t="s">
+      <c r="F26" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="G26" s="26" t="s">
+      <c r="G26" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="H26" s="26" t="s">
+      <c r="H26" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="I26" s="26" t="s">
+      <c r="I26" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="J26" s="26" t="s">
+      <c r="J26" s="14" t="s">
         <v>20</v>
       </c>
       <c r="K26" s="1"/>
@@ -2133,33 +2146,33 @@
       <c r="AK26" s="1"/>
     </row>
     <row r="27" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12" t="s">
+      <c r="A27" s="22"/>
+      <c r="B27" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D27" s="16">
+      <c r="D27" s="15">
         <v>1190.3</v>
       </c>
-      <c r="E27" s="16">
+      <c r="E27" s="15">
         <f>D27-D30</f>
         <v>4.7999999999999545</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G27" s="6">
+      <c r="G27" s="4">
         <v>0.06</v>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="4">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="4">
         <v>0.02</v>
       </c>
-      <c r="J27" s="14">
+      <c r="J27" s="27">
         <v>6.7999999999999996E-3</v>
       </c>
       <c r="K27" s="1"/>
@@ -2191,24 +2204,24 @@
       <c r="AK27" s="1"/>
     </row>
     <row r="28" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="18" t="s">
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="G28" s="18">
+      <c r="G28" s="11">
         <v>0.17</v>
       </c>
-      <c r="H28" s="18">
+      <c r="H28" s="11">
         <v>0.72</v>
       </c>
-      <c r="I28" s="18">
+      <c r="I28" s="11">
         <v>0.48</v>
       </c>
-      <c r="J28" s="15"/>
+      <c r="J28" s="28"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -2238,31 +2251,31 @@
       <c r="AK28" s="1"/>
     </row>
     <row r="29" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="9" t="s">
+      <c r="A29" s="22"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="4">
         <v>1194.4000000000001</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="4">
         <f>D29-D30</f>
         <v>8.9000000000000909</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="4">
         <v>-0.61</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="4">
         <v>0.185</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="4">
         <v>0.46</v>
       </c>
-      <c r="J29" s="6">
+      <c r="J29" s="4">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="K29" s="1"/>
@@ -2294,30 +2307,30 @@
       <c r="AK29" s="1"/>
     </row>
     <row r="30" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="10" t="s">
+      <c r="A30" s="22"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="5">
         <v>1185.5</v>
       </c>
-      <c r="E30" s="7">
+      <c r="E30" s="5">
         <v>0</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="5">
         <v>5.7000000000000002E-2</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H30" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I30" s="7">
+      <c r="I30" s="5">
         <v>0.02</v>
       </c>
-      <c r="J30" s="7">
+      <c r="J30" s="5">
         <v>6.7000000000000002E-3</v>
       </c>
       <c r="K30" s="1"/>
@@ -2349,30 +2362,30 @@
       <c r="AK30" s="1"/>
     </row>
     <row r="31" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="9" t="s">
+      <c r="A31" s="22"/>
+      <c r="B31" s="22"/>
+      <c r="C31" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="4">
         <v>1194.4000000000001</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="4">
         <v>8.9</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G31" s="8" t="s">
+      <c r="G31" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H31" s="8" t="s">
+      <c r="H31" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I31" s="8" t="s">
+      <c r="I31" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="J31" s="8" t="s">
+      <c r="J31" s="6" t="s">
         <v>20</v>
       </c>
       <c r="K31" s="1"/>
@@ -2561,12 +2574,16 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="E22:E23"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="J2:J3"/>
@@ -2583,16 +2600,835 @@
     <mergeCell ref="B17:B21"/>
     <mergeCell ref="B22:B26"/>
     <mergeCell ref="B27:B31"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J12:J13"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C22:C23"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B68326AF-0F6A-4F4A-8E87-CDE9E604DBA2}">
+  <dimension ref="A1:S34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="30">
+        <v>1765.7</v>
+      </c>
+      <c r="E2" s="30">
+        <v>-0.43</v>
+      </c>
+      <c r="F2" s="30">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="G2" s="30">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H2" s="30">
+        <v>1.4E-3</v>
+      </c>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="22"/>
+      <c r="B3" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="30">
+        <v>1765.7</v>
+      </c>
+      <c r="E3" s="30">
+        <v>-0.43</v>
+      </c>
+      <c r="F3" s="30">
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="G3" s="30">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="H3" s="30">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="22"/>
+      <c r="B4" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="30">
+        <v>1765.2</v>
+      </c>
+      <c r="E4" s="30">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="F4" s="30">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="G4" s="30">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="H4" s="30">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="29">
+        <v>1188.8</v>
+      </c>
+      <c r="E5" s="29">
+        <v>1.4E-2</v>
+      </c>
+      <c r="F5" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="29">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="H5" s="29">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="22"/>
+      <c r="B6" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="29">
+        <v>1188.5999999999999</v>
+      </c>
+      <c r="E6" s="29">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="F6" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" s="29">
+        <v>0.01</v>
+      </c>
+      <c r="H6" s="29">
+        <v>6.6E-3</v>
+      </c>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="22"/>
+      <c r="B7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="29">
+        <v>1185.5</v>
+      </c>
+      <c r="E7" s="29">
+        <v>5.7000000000000002E-2</v>
+      </c>
+      <c r="F7" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="29">
+        <v>0.02</v>
+      </c>
+      <c r="H7" s="29">
+        <v>6.7000000000000002E-3</v>
+      </c>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="R10" s="1"/>
+      <c r="S10" s="1"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
+      <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
+      <c r="R12" s="1"/>
+      <c r="S12" s="1"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1"/>
+      <c r="R13" s="1"/>
+      <c r="S13" s="1"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
+      <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="1"/>
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
+      <c r="R20" s="1"/>
+      <c r="S20" s="1"/>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1"/>
+      <c r="R21" s="1"/>
+      <c r="S21" s="1"/>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1"/>
+      <c r="R22" s="1"/>
+      <c r="S22" s="1"/>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+      <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
+      <c r="S27" s="1"/>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
+      <c r="R29" s="1"/>
+      <c r="S29" s="1"/>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
+      <c r="S34" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A7"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>